<commit_message>
actualiza acumulados 16/06/2026 18:45
</commit_message>
<xml_diff>
--- a/Pruebas calificadas/COLEGIO ARGELIA DIAGNOSTICAS 1102_CALIFICADO.xlsx
+++ b/Pruebas calificadas/COLEGIO ARGELIA DIAGNOSTICAS 1102_CALIFICADO.xlsx
@@ -8241,14 +8241,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V31" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V31" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W31" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X31" s="3" t="inlineStr">
@@ -8258,12 +8258,12 @@
       </c>
       <c r="Y31" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z31" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z31" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA31" s="2" t="inlineStr">
@@ -8494,14 +8494,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V32" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V32" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W32" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X32" s="3" t="inlineStr">
@@ -8511,12 +8511,12 @@
       </c>
       <c r="Y32" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z32" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z32" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA32" s="2" t="inlineStr">
@@ -8747,14 +8747,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V33" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V33" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W33" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X33" s="3" t="inlineStr">
@@ -8764,12 +8764,12 @@
       </c>
       <c r="Y33" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z33" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z33" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA33" s="2" t="inlineStr">
@@ -9000,9 +9000,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V34" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V34" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W34" s="2" t="inlineStr">
@@ -9253,14 +9253,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V35" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V35" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W35" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X35" s="3" t="inlineStr">
@@ -9270,12 +9270,12 @@
       </c>
       <c r="Y35" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z35" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z35" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA35" s="2" t="inlineStr">
@@ -9506,9 +9506,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V36" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V36" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W36" s="2" t="inlineStr">
@@ -9516,9 +9516,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="X36" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="X36" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="Y36" s="2" t="inlineStr">
@@ -9759,14 +9759,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V37" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V37" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W37" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X37" s="3" t="inlineStr">
@@ -9776,12 +9776,12 @@
       </c>
       <c r="Y37" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z37" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z37" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA37" s="2" t="inlineStr">
@@ -10012,14 +10012,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V38" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V38" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W38" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X38" s="3" t="inlineStr">
@@ -10029,12 +10029,12 @@
       </c>
       <c r="Y38" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z38" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z38" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA38" s="2" t="inlineStr">
@@ -10265,14 +10265,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V39" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V39" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W39" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X39" s="3" t="inlineStr">
@@ -10282,12 +10282,12 @@
       </c>
       <c r="Y39" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z39" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z39" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA39" s="2" t="inlineStr">
@@ -10518,14 +10518,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V40" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V40" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W40" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="X40" s="3" t="inlineStr">
@@ -10535,7 +10535,7 @@
       </c>
       <c r="Y40" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="Z40" s="3" t="inlineStr">
@@ -10771,14 +10771,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V41" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V41" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W41" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X41" s="3" t="inlineStr">
@@ -10788,12 +10788,12 @@
       </c>
       <c r="Y41" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z41" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z41" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA41" s="2" t="inlineStr">
@@ -11024,14 +11024,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V42" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V42" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W42" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X42" s="3" t="inlineStr">
@@ -11041,12 +11041,12 @@
       </c>
       <c r="Y42" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z42" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Z42" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA42" s="2" t="inlineStr">
@@ -11273,14 +11273,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V43" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V43" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W43" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X43" s="3" t="inlineStr">
@@ -11290,12 +11290,12 @@
       </c>
       <c r="Y43" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z43" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z43" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA43" s="2" t="inlineStr">
@@ -11526,14 +11526,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V44" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V44" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W44" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X44" s="3" t="inlineStr">
@@ -11543,12 +11543,12 @@
       </c>
       <c r="Y44" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z44" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z44" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA44" s="2" t="inlineStr">
@@ -11779,14 +11779,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V45" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V45" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W45" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X45" s="3" t="inlineStr">
@@ -11796,12 +11796,12 @@
       </c>
       <c r="Y45" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z45" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z45" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA45" s="2" t="inlineStr">
@@ -12039,7 +12039,7 @@
       </c>
       <c r="W46" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X46" s="3" t="inlineStr">
@@ -12049,12 +12049,12 @@
       </c>
       <c r="Y46" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z46" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Z46" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA46" s="2" t="inlineStr">
@@ -12285,29 +12285,29 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V47" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V47" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W47" s="2" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X47" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="Y47" s="2" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="X47" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
-        </is>
-      </c>
-      <c r="Y47" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z47" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+      <c r="Z47" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA47" s="2" t="inlineStr">
@@ -12538,14 +12538,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V48" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V48" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W48" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X48" s="3" t="inlineStr">
@@ -12555,12 +12555,12 @@
       </c>
       <c r="Y48" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z48" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Z48" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA48" s="2" t="inlineStr">
@@ -12791,29 +12791,29 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V49" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V49" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W49" s="2" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X49" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="Y49" s="2" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="X49" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
-        </is>
-      </c>
-      <c r="Y49" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z49" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+      <c r="Z49" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA49" s="2" t="inlineStr">
@@ -13044,29 +13044,29 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V50" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V50" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W50" s="2" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X50" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="Y50" s="2" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="X50" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
-        </is>
-      </c>
-      <c r="Y50" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z50" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+      <c r="Z50" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA50" s="2" t="inlineStr">
@@ -13297,14 +13297,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V51" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V51" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W51" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X51" s="3" t="inlineStr">
@@ -13314,12 +13314,12 @@
       </c>
       <c r="Y51" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z51" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z51" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA51" s="2" t="inlineStr">
@@ -13550,29 +13550,29 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V52" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V52" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W52" s="2" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X52" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="Y52" s="2" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="X52" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
-        </is>
-      </c>
-      <c r="Y52" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z52" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+      <c r="Z52" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA52" s="2" t="inlineStr">
@@ -13803,29 +13803,29 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V53" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V53" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W53" s="2" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X53" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="Y53" s="2" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="X53" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
-        </is>
-      </c>
-      <c r="Y53" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z53" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+      <c r="Z53" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA53" s="2" t="inlineStr">
@@ -14056,14 +14056,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V54" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V54" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W54" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X54" s="3" t="inlineStr">
@@ -14073,12 +14073,12 @@
       </c>
       <c r="Y54" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z54" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Z54" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA54" s="2" t="inlineStr">
@@ -14309,14 +14309,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V55" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V55" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W55" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X55" s="3" t="inlineStr">
@@ -14326,12 +14326,12 @@
       </c>
       <c r="Y55" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z55" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z55" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA55" s="2" t="inlineStr">
@@ -14562,14 +14562,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V56" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V56" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W56" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X56" s="3" t="inlineStr">
@@ -14579,12 +14579,12 @@
       </c>
       <c r="Y56" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z56" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z56" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA56" s="2" t="inlineStr">
@@ -14815,14 +14815,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V57" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V57" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W57" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X57" s="3" t="inlineStr">
@@ -14832,12 +14832,12 @@
       </c>
       <c r="Y57" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z57" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z57" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA57" s="2" t="inlineStr">
@@ -15068,14 +15068,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V58" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V58" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W58" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X58" s="3" t="inlineStr">
@@ -15085,12 +15085,12 @@
       </c>
       <c r="Y58" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z58" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z58" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA58" s="2" t="inlineStr">
@@ -15321,14 +15321,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V59" s="3" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V59" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W59" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X59" s="3" t="inlineStr">
@@ -15338,12 +15338,12 @@
       </c>
       <c r="Y59" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Z59" s="4" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z59" s="3" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AA59" s="2" t="inlineStr">

</xml_diff>